<commit_message>
Add item weights and shipping tab to Michigan Box workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SS8EsZNZJgzhYPJLGv3Rn9
</commit_message>
<xml_diff>
--- a/Michigan_Box_By_Item.xlsx
+++ b/Michigan_Box_By_Item.xlsx
@@ -8,14 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Cherries" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Fudge" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Cream-Nut" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Peanuts" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Pretzels" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Kars" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Faygo" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Card" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shipping" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Cherries" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Fudge" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Cream-Nut" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Peanuts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Pretzels" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Kars" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Faygo" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Card" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -71,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -79,6 +80,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -457,6 +461,7 @@
     <col width="52" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="60" customHeight="1">
@@ -517,6 +522,11 @@
           <t>Est. price (cheapest option)</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Est. item weight (with its own packaging)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -555,6 +565,11 @@
           <t>Germack 8 oz $14.24 (online/store)</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>8.4 oz (8 oz net)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -595,6 +610,11 @@
           <t>Joann’s Five Slice Box $46.95 ≈ $9.39/slice</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>9.0 oz (8 oz net)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -640,6 +660,11 @@
           <t>Koeze 6-jar case $41.95 ≈ $6.99/jar</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>26.5 oz (17 oz net)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -678,6 +703,11 @@
           <t>Germack 10 lb bulk $24.99 ≈ $1.40 per 9 oz (7 oz bag $4.25)</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>9.4 oz (9 oz net)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -721,6 +751,11 @@
           <t>Single bags ~$4.79–$5 (skip the $100 case)</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>8.0 oz (7.5 oz net)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -769,6 +804,11 @@
           <t>Sam’s Club 40-pk $17.48 ≈ $0.44/bag</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2.2 oz (2 oz net)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -812,6 +852,11 @@
           <t>In-store Kroger/Meijer 12-pack (skip online ~$24)</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>13.0 oz (12 fl oz net)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -848,6 +893,416 @@
       <c r="J10" t="inlineStr">
         <is>
           <t>Custom print run (get quotes)</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1.0 oz (5×7 in net)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="60" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Greetings from Detroit card, 5 × 7. Paper Source is the closest blank-card option. For cards by Detroit artists, or a custom printed run, go to Detroit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Place</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Miles from Birmingham</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Est. price</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paper Source</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>115 W Maple Rd, Birmingham</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Stationery (chain)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Listed</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Blank 5×7 cards and envelopes.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://birmingham-mi.yiftee.com/business/paper-source-473129</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>~$5–$8 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Write Impressions</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Royal Oak</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Stationery</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Listed</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Stationery shop since 1989.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>~$5–$8 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>City Bird</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>460 W Canfield St, Detroit</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>313-831-9146</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Local-artist shop</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>100+ Detroit/Michigan-themed cards.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://visitdetroit.com/directory/city-bird/</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>~$5–$8 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Signal Return (letterpress)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Kercheval Ave, Detroit (verify)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Custom printing</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Listed</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Custom letterpress cards.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Vesey Lane Goods</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>9920 Kercheval Ave, Detroit</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Local makers</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Listed</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>~$5–$8 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pure Detroit</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>70 W Alexandrine St, Detroit</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Detroit goods</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Listed</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>~$5–$8 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Pack size</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Per unit</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Custom printed run (letterpress/print shop)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>per quote</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>get quotes</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Likely cheapest per card at volume; no prices found</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Paper Source / City Bird single cards</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>in store</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No prices found online</t>
         </is>
       </c>
     </row>
@@ -860,6 +1315,382 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Shipping weight and box. Weights are estimates; weigh one packed box on a postal scale and enter that number in your label software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Net weight</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Est. weight w/ own packaging (oz)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Approx. size</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Germack Dried Cherries</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>8 oz</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>flat bag ~6×9×1.5 in</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mackinac Island Fudge slab</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>8 oz</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>wrapped slab ~5×3×1 in</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Freezes and is heat-sensitive: avoid hot trucks in summer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Koeze Cream-Nut (glass jar)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>17 oz</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>jar ~3.3 in dia × 4.6 in tall</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Glass jar is the heaviest item. Wrap it and keep it centered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Germack In-Shell Peanuts</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>9 oz</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>bag ~6×10×2.5 in</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pop Daddy Dill Pickle Pretzels</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7.5 oz</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>bag ~7×11×2.5 in (puffy)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kar’s Sweet ’N Salty</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2 oz</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>bag ~4×6 in</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Faygo Rock &amp; Rye can</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>12 fl oz</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>can 2.6 in dia × 4.8 in</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Can may burst if it freezes (Nov–Mar). Bag it in case it leaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Greetings from Detroit card + envelope</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>5×7 in</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>5.25×7.25 in</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Contents subtotal</t>
+        </is>
+      </c>
+      <c r="C12">
+        <f>SUM(C4:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>≈ 4.8 lb</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gift box + shipping box + filler (est.)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>20</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>≈ 1–1.5 lb, depends on your box</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ESTIMATED TOTAL SHIPPED WEIGHT</t>
+        </is>
+      </c>
+      <c r="C14">
+        <f>C12+C13</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>ROUND(C14/16,1)&amp;" lb"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>BOX SIZE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sample box in your label tool</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>8.6 × 5.4 × 1.6 in</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Too small: the jar and can alone are taller than 1.6 in</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Suggested shipping box</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>12 × 10 × 6 in (or 12 × 9 × 6)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Fits a gift box with all 8 items plus filler</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Dimensional weight (UPS/FedEx, ÷139)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>12×10×6 = 720 in³ ÷ 139 ≈ 5.2 lb</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Lower than the actual ~6.1 lb, so you are billed on actual weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>USPS Ground Advantage</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Dim weight only applies over 1 cu ft (1,728 in³)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Billed on actual weight, rounded up to the next lb (≈ 7 lb)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Enter in label tool</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Box, 12 × 10 × 6 in, total ≈ 6.1 lb (confirm on a scale)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Then re-check rates. The $6.70 quote was based on 3.6 lb.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2676,7 +3507,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
@@ -2756,7 +3586,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3139,7 +3969,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -3337,7 +4166,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3696,7 +4525,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -3867,7 +4695,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4423,7 +5251,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -4535,7 +5362,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6068,7 +6895,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
@@ -6239,7 +7065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6752,7 +7578,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -6940,7 +7765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7514,7 +8339,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
@@ -7610,412 +8434,6 @@
       <c r="G21" t="inlineStr">
         <is>
           <t>https://www.walmart.com/ip/seort/631284437</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="60" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Greetings from Detroit card, 5 × 7. Paper Source is the closest blank-card option. For cards by Detroit artists, or a custom printed run, go to Detroit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Place</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Address</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Miles from Birmingham</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Confidence</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Est. price</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paper Source</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>115 W Maple Rd, Birmingham</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Stationery (chain)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Listed</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Blank 5×7 cards and envelopes.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://birmingham-mi.yiftee.com/business/paper-source-473129</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>~$5–$8 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Write Impressions</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Royal Oak</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Stationery</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Listed</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Stationery shop since 1989.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>~$5–$8 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>City Bird</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>460 W Canfield St, Detroit</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>15.8</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>313-831-9146</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Local-artist shop</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>100+ Detroit/Michigan-themed cards.</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://visitdetroit.com/directory/city-bird/</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>~$5–$8 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Signal Return (letterpress)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Kercheval Ave, Detroit (verify)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Custom printing</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Listed</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Custom letterpress cards.</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Quote</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Vesey Lane Goods</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>9920 Kercheval Ave, Detroit</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Local makers</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Listed</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>~$5–$8 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Pure Detroit</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>70 W Alexandrine St, Detroit</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Detroit goods</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Listed</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>~$5–$8 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Option</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Pack size</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Per unit</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Custom printed run (letterpress/print shop)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>per quote</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>get quotes</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Likely cheapest per card at volume; no prices found</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Paper Source / City Bird single cards</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>in store</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>No prices found online</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Highlight places that appear across multiple item tabs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SS8EsZNZJgzhYPJLGv3Rn9
</commit_message>
<xml_diff>
--- a/Michigan_Box_By_Item.xlsx
+++ b/Michigan_Box_By_Item.xlsx
@@ -42,7 +42,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,11 @@
         <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9C2F0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -72,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -83,6 +88,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,7 +473,7 @@
     <row r="1" ht="60" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Michigan Box: one tab per item, sorted nearest to Birmingham, MI (48009) first. Stockist rows come from the brands’ official store locators (pulled 10/26/2026). Those list stores carrying the brand, not the exact bag, so call ahead. Prices come from public listings and may change. Each item tab ends with a PRICE COMPARISON table (cheapest first, highlighted green). "Est. price" = a price found in a listing, or "(est.)" where it is an estimate. Confirm in store.</t>
+          <t>The Michigan Box: one tab per item, sorted nearest to Birmingham, MI (48009) first. Stockist rows come from the brands’ official store locators (pulled 10/26/2026). Those list stores carrying the brand, not the exact bag, so call ahead. Prices come from public listings and may change. Each item tab ends with a PRICE COMPARISON table (cheapest first, highlighted green). "Est. price" = a price found in a listing, or "(est.)" where it is an estimate. Confirm in store. PURPLE rows = the same place appears in 2+ other item tabs (one stop for several items).</t>
         </is>
       </c>
     </row>
@@ -1213,6 +1219,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -1383,7 +1390,6 @@
           <t>flat bag ~6×9×1.5 in</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1454,7 +1460,6 @@
           <t>bag ~6×10×2.5 in</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1475,7 +1480,6 @@
           <t>bag ~7×11×2.5 in (puffy)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1496,7 +1500,6 @@
           <t>bag ~4×6 in</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1542,7 +1545,6 @@
           <t>5.25×7.25 in</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1907,109 +1909,116 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Beverage Warehouse</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>31111 Greenfield, Beverly Hills MI 48009</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Market Square #1 - Birmingham</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>1964 Southfield Rd, Birmingham MI 48009</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Also Pop Daddy</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Market Square (former Papa Joe’s)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>34244 Woodward, Birmingham MI 48009</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Also Pop Daddy</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
@@ -2049,104 +2058,112 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Troy Cheese &amp; Wine Barn</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>2558 E. Maple, Troy MI 48084</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Market Fresh - Bev Hills</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>31201 Southfield, Beverly Hills MI 48025</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="6" t="n">
         <v>2.7</v>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Also Pop Daddy</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>BLOOMFIELD MOBIL</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="6" t="n">
         <v>3.1</v>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
@@ -2252,71 +2269,76 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Westborn Market - Berkley</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>27659 Woodward Rd., Berkley MI 48072</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="6" t="n">
         <v>3.2</v>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Also Pop Daddy</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Campbell Party Store</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>3321 Campbell, Royal Oak MI 48073</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="6" t="n">
         <v>3.4</v>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
@@ -2389,33 +2411,36 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>MOBIL - TELEGRAPH</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>6490 TELEGRAPH RD, BLOOMFIELD HILLS MI 48301</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
@@ -2455,109 +2480,116 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Plum Market</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>3675 W Maple, Bloomfield Hills MI 48301</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Also Pop Daddy</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Plum Market - Bloomfield Hills</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>3675 W Maple, Bloomfield Hills MI 48301</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Also Pop Daddy</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Shell _Bloomfield - Barbat</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>3690 W Maple, West Bloomfiled MI 48301</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
@@ -2597,66 +2629,72 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Manny's Liquor</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>42951 Dequindre, Troy MI 48098</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D26" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="6" t="n"/>
+      <c r="J26" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Bloomfield Wine &amp; Spirits</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>1081 W. Long Lake Road, Bloomfield Hills MI 48302</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="6" t="n"/>
+      <c r="J27" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
@@ -2762,38 +2800,40 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Hollywood Market #2 - Royal Oak</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>714 Main Street, Royal Oak MI 48067</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="6" t="n">
         <v>5.4</v>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Also Pop Daddy</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="I31" s="6" t="n"/>
+      <c r="J31" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
@@ -3031,66 +3071,72 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Nino Salvaggio's</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>6835 Rochester Rd., Troy MI 48085</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D39" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
+      <c r="E39" s="6" t="n"/>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="6" t="n"/>
+      <c r="J39" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Nino Salvaggio's - Troy</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>6835 Rochester Rd., Troy MI 48085</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D40" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="6" t="n"/>
+      <c r="J40" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
@@ -3130,76 +3176,80 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Hollywood Market</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>29200 N Campbell, Madison Heights MI 48071</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D42" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>Also Pop Daddy</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="I42" s="6" t="n"/>
+      <c r="J42" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Hollywood Market #1</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>29200 N Campbell, Madison Heights MI 48071</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D43" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>Also Pop Daddy</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="I43" s="6" t="n"/>
+      <c r="J43" s="6" t="inlineStr">
         <is>
           <t>~$12–$16 (est.)</t>
         </is>
@@ -3507,6 +3557,7 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
@@ -3969,6 +4020,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -4247,76 +4299,80 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Kroger</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>685 E Maple Rd, Birmingham</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Grocery (check)</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Possible</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Search “Cream-Nut” on kroger.com with this store selected.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>~$7–$8 (est.)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Kroger</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>1237 Coolidge Hwy, Troy</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Grocery (check)</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Possible</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Same check.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>~$7–$8 (est.)</t>
         </is>
@@ -4525,6 +4581,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -4872,114 +4929,120 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Beverage Warehouse</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>31111 Greenfield, Beverly Hills MI 48009</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>See tab 1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>~$4–$6 (est.)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Market Square #1 - Birmingham</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>1964 Southfield Rd, Birmingham MI 48009</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>See tab 1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>~$4–$6 (est.)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Market Square (former Papa Joe’s)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>34244 Woodward, Birmingham MI 48009</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>See tab 1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>~$4–$6 (est.)</t>
         </is>
@@ -5024,114 +5087,120 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Troy Cheese &amp; Wine Barn</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>2558 E. Maple, Troy MI 48084</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>See tab 1</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>~$4–$6 (est.)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Market Fresh - Bev Hills</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>31201 Southfield, Beverly Hills MI 48025</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="6" t="n">
         <v>2.7</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>See tab 1</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>~$4–$6 (est.)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>BLOOMFIELD MOBIL</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="6" t="n">
         <v>3.1</v>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Germack locator</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>See tab 1</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>~$4–$6 (est.)</t>
         </is>
@@ -5251,6 +5320,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -5488,152 +5558,160 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Market Square (former Papa Joe’s)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>34244 Woodward Ave, Birmingham, MI 48009</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>10 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Mkt Square(Birm)Special</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>1964 Southfield Rd, Birmingham, MI 48009</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>6 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>KROGER</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>685 E Maple Road, Birmingham, MI 48009</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>4 PD items</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>KROGER</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>1237 Coolidge Highway, Troy, MI 48084</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>4 PD items</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -5721,38 +5799,40 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Mkt Fresh</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>31201 Southfield Rd, Beverly hills, MI 48025</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="6" t="n">
         <v>2.7</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>6 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -5797,43 +5877,44 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Westborn Market</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>27659 Woodward Avenue, Berkley, MI 48072</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="6" t="n">
         <v>3.2</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>(248) 547-1000</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>13 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -5878,38 +5959,40 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Westborn(Berk)Grocery</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>27659 Woodward Ave, Berkley, MI 48072</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="6" t="n">
         <v>3.2</v>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>1 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -5992,43 +6075,44 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Plum Market</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>3675 West Maple Road, Bloomfield township, MI 48301</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>(248) 594-2555</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>16 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -6073,38 +6157,40 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Nino's (Troy) - Grocery</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>6835 Rochester Rd, Troy, MI 48098</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>3 PD items</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -6187,81 +6273,84 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Hollywood Markets</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>714 N Main Street, Royal oak, MI 48067</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" s="6" t="n">
         <v>5.4</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>(248) 548-5051</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>10 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Hollywood</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>714 N. Main, Royal oak, MI 48067</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" s="6" t="n">
         <v>5.4</v>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>7 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -6420,81 +6509,84 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Hollywood Markets</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>29200 North Campbell Road, Madison heights, MI 48071</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>(248) 399-0900</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>8 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="I28" s="6" t="n"/>
+      <c r="J28" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Hollywood</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>29200 Campbell Rd, Madison heights, MI 48071</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>6 PD items · also Germack</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="I29" s="6" t="n"/>
+      <c r="J29" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -6895,6 +6987,7 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
@@ -7194,38 +7287,40 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Kroger</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>685 E Maple Rd, Birmingham</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Grocery</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Single bags.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>~$1–$1.50 (est.)</t>
         </is>
@@ -7315,269 +7410,294 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Beverage Warehouse</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>31111 Greenfield, Beverly Hills MI 48009</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Troy Cheese &amp; Wine Barn</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>2558 E. Maple, Troy MI 48084</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>BLOOMFIELD MOBIL</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="6" t="n">
         <v>3.1</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Campbell Party Store</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>3321 Campbell, Royal Oak MI 48073</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="6" t="n">
         <v>3.4</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>MOBIL - TELEGRAPH</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>6490 TELEGRAPH RD, BLOOMFIELD HILLS MI 48301</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Shell _Bloomfield - Barbat</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>3690 W Maple, West Bloomfiled MI 48301</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Manny's Liquor</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>42951 Dequindre, Troy MI 48098</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Bloomfield Wine &amp; Spirits</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>1081 W. Long Lake Road, Bloomfield Hills MI 48302</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -7846,33 +7966,36 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Kroger</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>685 E Maple Rd, Birmingham</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Grocery</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>~$1–$1.25/can in 12-pk (est.)</t>
         </is>
@@ -7965,33 +8088,36 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Kroger</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>1237 Coolidge Hwy, Troy</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Grocery</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>~$1–$1.25/can in 12-pk (est.)</t>
         </is>
@@ -8076,269 +8202,294 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Beverage Warehouse</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>31111 Greenfield, Beverly Hills MI 48009</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>~$1.50–$2.50/can (est.)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Troy Cheese &amp; Wine Barn</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>2558 E. Maple, Troy MI 48084</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>~$1.50–$2.50/can (est.)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>BLOOMFIELD MOBIL</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="6" t="n">
         <v>3.1</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>~$1.50–$2.50/can (est.)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Campbell Party Store</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>3321 Campbell, Royal Oak MI 48073</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="6" t="n">
         <v>3.4</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>~$1.50–$2.50/can (est.)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>MOBIL - TELEGRAPH</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>6490 TELEGRAPH RD, BLOOMFIELD HILLS MI 48301</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>~$1.50–$2.50/can (est.)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Shell _Bloomfield - Barbat</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>3690 W Maple, West Bloomfiled MI 48301</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>~$1.50–$2.50/can (est.)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Manny's Liquor</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>42951 Dequindre, Troy MI 48098</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>~$1.50–$2.50/can (est.)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Bloomfield Wine &amp; Spirits</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>1081 W. Long Lake Road, Bloomfield Hills MI 48302</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Party store</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>~$1.50–$2.50/can (est.)</t>
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Ace Hardware (Devon's Mackinac Island Fudge) as nearby fudge source
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SS8EsZNZJgzhYPJLGv3Rn9
</commit_message>
<xml_diff>
--- a/Michigan_Box_By_Item.xlsx
+++ b/Michigan_Box_By_Item.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -588,8 +588,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Order direct from Murdick’s / Ryba’s / Joann’s</t>
-        </is>
+          <t>Ace Hardware, 17670 13 Mile Rd, Beverly Hills (Devon’s Mackinac Island Fudge)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2.7</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -598,22 +601,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Ship</t>
+          <t>Best nearby stop</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Ace sells Devon’s; call to confirm</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>No Birmingham retailer confirmed; check the lead at 1540 W Lincoln, Birmingham</t>
+          <t>7 oz tub. Clawson, Southfield and Royal Oak Aces too. Ship from Joann’s if none in stock.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Joann’s Five Slice Box $46.95 ≈ $9.39/slice</t>
+          <t>$4.99 (7 oz tub)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -907,6 +910,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
@@ -1219,7 +1223,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -3557,7 +3560,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
@@ -3643,7 +3645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3661,7 +3663,7 @@
     <row r="1" ht="60" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Mackinac Island Fudge, 8 oz slab. No Birmingham retailer is confirmed. Island makers sell half-pound (≈8 oz) slices and ship.</t>
+          <t>Mackinac Island Fudge. Any brand labeled “Mackinac Island Fudge” works. CLOSEST AND CHEAPEST (green): Ace Hardware stores carry Devon’s Mackinac Island Fudge, 7 oz tubs, $4.99 on acehardware.com. That’s 7 oz, not an 8 oz slab. In-store stock varies, so call ahead. Otherwise order half-pound slices from the island makers below.</t>
         </is>
       </c>
     </row>
@@ -3718,185 +3720,178 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>“Original Murdicks Fudge” address (LEAD)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1540 W Lincoln, Birmingham 48009</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>(906) 643-9616</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Lead</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Unverified</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Listed under Murdick’s name on Germack’s stockist list. No storefront found; may be an office. Ask Murdick’s about local pickup or bulk.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://www.originalmurdicksfudge.com/about-us/</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Ask</t>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Ace Hardware – Beverly Hills</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>17670 13 Mile Rd, Beverly Hills 48025</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Retail (Ace)</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Ace sells Devon’s online</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Devon’s Mackinac Island Fudge 7 oz tub. Also on Germack’s stockist list. Call to confirm in stock.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.acehardware.com/p/9047289</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>$4.99 (7 oz)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Original Murdick’s Fudge</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Mackinac Island / Mackinaw City / St. Ignace</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>(906) 847-3530 · business (906) 643-9616</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Ship</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Half-pound slices. Single Slice Box $15.95, Three Slice $41.95. Ships US via FedEx. Corporate and group sales.</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>https://www.originalmurdicksfudge.com</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>$13.98–$15.95/slice</t>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Great Lakes Ace Hardware – Clawson</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>149 E 14 Mile Rd, Clawson 48017</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Retail (Ace)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Ace sells Devon’s online</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Same: Devon’s 7 oz tubs; also a Germack stockist.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.acehardware.com/p/9047289</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>$4.99 (7 oz)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Ryba’s Mackinac Island Fudge</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Mackinac Island</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>800-447-9227 · info@ryba.com</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Ship</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Shipping restarts the week of 11/2 after the off-season move. Free shipping over $99. Corporate gifting.</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://ryba.com</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>≈ $11.98/slice</t>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Great Lakes Ace Hardware – Southfield</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>29201 Greenfield Rd, Southfield 48076</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Retail (Ace)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Ace sells Devon’s online</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Same.</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.acehardware.com/p/9047289</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>$4.99 (7 oz)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Joann’s Fudge</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Mackinac Island; 303 E Central, Mackinaw City</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>906-847-6357</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Ship</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>One Slice Box $12.95; corporate gifts.</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>https://www.joannsfudge.com</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>$9.39–$12.95/slice</t>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Great Lakes Ace Hardware – Royal Oak</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>515 E 4th St, Royal Oak 48067</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Retail (Ace)</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Ace sells Devon’s online</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Same.</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.acehardware.com/p/9047289</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>$4.99 (7 oz)</t>
         </is>
       </c>
     </row>
@@ -3906,42 +3901,45 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Original Mackinac Island Fudge Co.</t>
+          <t>“Original Murdicks Fudge” address (LEAD)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Online (Michigan-Made)</t>
-        </is>
+          <t>1540 W Lincoln, Birmingham 48009</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>via contact page</t>
+          <t>(906) 643-9616</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>Unverified</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Says it offers wholesale; use the request form.</t>
+          <t>Listed under Murdick’s name on Germack’s stockist list. No storefront found; may be an office. Ask Murdick’s about local pickup or bulk.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://michigan-made.com/shop/wholesale/</t>
+          <t>https://www.originalmurdicksfudge.com/about-us/</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Wholesale (ask)</t>
+          <t>Ask</t>
         </is>
       </c>
     </row>
@@ -3951,37 +3949,42 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Devon’s Mackinac Island Fudge</t>
+          <t>Original Murdick’s Fudge</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>St. Ignace</t>
+          <t>Mackinac Island / Mackinaw City / St. Ignace</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>(906) 847-3530 · business (906) 643-9616</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Wholesale (Faire)</t>
+          <t>Ship</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Listed</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Mostly 5.5 oz; $144 minimum.</t>
+          <t>Half-pound slices. Single Slice Box $15.95, Three Slice $41.95. Ships US via FedEx. Corporate and group sales.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://www.faire.com/brand/b_6x2vvtmhv4</t>
+          <t>https://www.originalmurdicksfudge.com</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>~$12.95 per 5.5 oz</t>
+          <t>$13.98–$15.95/slice</t>
         </is>
       </c>
     </row>
@@ -3991,220 +3994,395 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Ryba’s Mackinac Island Fudge</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mackinac Island</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>800-447-9227 · info@ryba.com</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Ship</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Shipping restarts the week of 11/2 after the off-season move. Free shipping over $99. Corporate gifting.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://ryba.com</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>≈ $11.98/slice</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Joann’s Fudge</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mackinac Island; 303 E Central, Mackinaw City</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>906-847-6357</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Ship</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>One Slice Box $12.95; corporate gifts.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.joannsfudge.com</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>$9.39–$12.95/slice</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Original Mackinac Island Fudge Co.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Online (Michigan-Made)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>via contact page</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Reported</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Says it offers wholesale; use the request form.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://michigan-made.com/shop/wholesale/</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Wholesale (ask)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Devon’s Mackinac Island Fudge</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>St. Ignace</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Wholesale (Faire)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Listed</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Mostly 5.5 oz; $144 minimum.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.faire.com/brand/b_6x2vvtmhv4</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>~$12.95 per 5.5 oz</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>Hefling’s Amish Farm Market</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Clinton Township</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Unverified</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>A Yelp review says it carries Mackinac fudge.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>~$10–$16 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="2" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Pack size</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Per unit</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="4" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Joann’s Five Slice Box</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>5 slices (½ lb each)</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>$46.95</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>≈ $9.39/slice</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>CHEAPEST + shipping</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>https://www.joannsfudge.com</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" t="inlineStr">
+    <row r="18">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Ryba’s Fudge Trio</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>3 slices</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>$35.95</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>≈ $11.98/slice</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Slice weight not stated; free shipping over $99</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>https://ryba.com</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" t="inlineStr">
+    <row r="19">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Joann’s One Slice Box</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>1 slice</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>$12.95</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>$12.95/slice</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>https://www.joannsfudge.com</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" t="inlineStr">
+    <row r="20">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Murdick’s Three Slice Box</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>3 × ½ lb</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>$41.95</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>≈ $13.98/slice</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>https://www.originalmurdicksfudge.com</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" t="inlineStr">
+    <row r="21">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Murdick’s Single Slice Box</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>1 × ½ lb</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>$15.95</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>$15.95/slice</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Most expensive</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>https://www.originalmurdicksfudge.com</t>
         </is>
@@ -4581,7 +4759,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -5320,7 +5497,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -6987,7 +7163,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
@@ -7697,7 +7872,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -8489,7 +8663,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Meijer Royal Oak (Cream-Nut, Faygo, Pop Daddy) to workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SS8EsZNZJgzhYPJLGv3Rn9
</commit_message>
<xml_diff>
--- a/Michigan_Box_By_Item.xlsx
+++ b/Michigan_Box_By_Item.xlsx
@@ -473,7 +473,7 @@
     <row r="1" ht="60" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Michigan Box: one tab per item, sorted nearest to Birmingham, MI (48009) first. Stockist rows come from the brands’ official store locators (pulled 10/26/2026). Those list stores carrying the brand, not the exact bag, so call ahead. Prices come from public listings and may change. Each item tab ends with a PRICE COMPARISON table (cheapest first, highlighted green). "Est. price" = a price found in a listing, or "(est.)" where it is an estimate. Confirm in store. PURPLE rows = the same place appears in 2+ other item tabs (one stop for several items).</t>
+          <t>The Michigan Box: one tab per item, sorted nearest to Birmingham, MI (48009) first. Stockist rows come from the brands’ official store locators (pulled 10/26/2026). Those list stores carrying the brand, not the exact bag, so call ahead. Prices come from public listings and may change. Each item tab ends with a PRICE COMPARISON table (cheapest first, highlighted green). "Est. price" = a price found in a listing, or "(est.)" where it is an estimate. Confirm in store. PURPLE rows = the same place appears in 2+ other item tabs (one stop for several items). Meijer Royal Oak (5150 Coolidge Hwy) added: confirmed online for Cream-Nut and Faygo Rock &amp; Rye.</t>
         </is>
       </c>
     </row>
@@ -636,8 +636,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Koeze direct 6-jar case ($41.95)</t>
-        </is>
+          <t>Meijer, 5150 Coolidge Hwy, Royal Oak (listed on meijer.com)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -646,12 +649,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Ship</t>
+          <t>Best nearby stop</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>On meijer.com</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -666,7 +669,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Koeze 6-jar case $41.95 ≈ $6.99/jar</t>
+          <t>$7.49 ($5.99 sale)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -4198,7 +4201,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -4402,7 +4404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4482,37 +4484,45 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Kroger</t>
+          <t>Meijer – Royal Oak</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>685 E Maple Rd, Birmingham</t>
+          <t>5150 Coolidge Hwy, Royal Oak 48073</t>
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E3" s="6" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>(248) 280-1800</t>
+        </is>
+      </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Grocery (check)</t>
+          <t>Grocery</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Possible</t>
+          <t>On meijer.com</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Search “Cream-Nut” on kroger.com with this store selected.</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="n"/>
+          <t>Cream-Nut Natural Smooth 17 oz listed on meijer.com. Open 6 AM–midnight. Check the app for store stock.</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>https://www.meijer.com/shopping/product/cream-nut-natural-smooth-peanut-butter-17-oz/7115730341.html</t>
+        </is>
+      </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>~$7–$8 (est.)</t>
+          <t>$7.49 ($5.99 on sale)</t>
         </is>
       </c>
     </row>
@@ -4527,11 +4537,11 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>1237 Coolidge Hwy, Troy</t>
+          <t>685 E Maple Rd, Birmingham</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>1.9</v>
+        <v>0.2</v>
       </c>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="inlineStr">
@@ -4546,7 +4556,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Same check.</t>
+          <t>Search “Cream-Nut” on kroger.com with this store selected.</t>
         </is>
       </c>
       <c r="I4" s="6" t="n"/>
@@ -4557,38 +4567,40 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Kroger</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>3600 W Maple Rd, Bloomfield Hills</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>1237 Coolidge Hwy, Troy</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Grocery (check)</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Possible</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Same check.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>~$7–$8 (est.)</t>
         </is>
@@ -4600,42 +4612,35 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Koeze direct – 6-jar case</t>
+          <t>Kroger</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ships from Grand Rapids</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>(616) 724-2620</t>
-        </is>
+          <t>3600 W Maple Rd, Bloomfield Hills</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3.5</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Ship</t>
+          <t>Grocery (check)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Possible</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Six 17 oz jars, $41.95 sale ($47.95 regular). Can ship to multiple addresses.</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>https://koeze.com/cream-nut-smooth-case-small</t>
+          <t>Same check.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>≈ $6.99/jar</t>
+          <t>~$7–$8 (est.)</t>
         </is>
       </c>
     </row>
@@ -4645,17 +4650,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Koeze business / bulk orders</t>
+          <t>Koeze direct – 6-jar case</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Ships from Grand Rapids</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>(616) 724-2620</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Wholesale</t>
+          <t>Ship</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4665,17 +4675,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Corporate gifts page, or contact for large orders.</t>
+          <t>Six 17 oz jars, $41.95 sale ($47.95 regular). Can ship to multiple addresses.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://koeze.com/gifts/corporate</t>
+          <t>https://koeze.com/cream-nut-smooth-case-small</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Wholesale (ask)</t>
+          <t>≈ $6.99/jar</t>
         </is>
       </c>
     </row>
@@ -4685,22 +4695,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Zingerman’s Deli</t>
+          <t>Koeze business / bulk orders</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>422 Detroit St, Ann Arbor</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>(734) 663-3354</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Retail + mail order</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4710,17 +4715,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Carries Cream-Nut.</t>
+          <t>Corporate gifts page, or contact for large orders.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://www.zingermans.com/Product/koeze-cream-nut-peanut-butter/P-BUT</t>
+          <t>https://koeze.com/gifts/corporate</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>~$8–$10 (est.)</t>
+          <t>Wholesale (ask)</t>
         </is>
       </c>
     </row>
@@ -4730,142 +4735,156 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Zingerman’s Deli</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>422 Detroit St, Ann Arbor</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>(734) 663-3354</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Retail + mail order</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Carries Cream-Nut.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.zingermans.com/Product/koeze-cream-nut-peanut-butter/P-BUT</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>~$8–$10 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>Koeze stores</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>2577 Burlingame Ave SW / 1971 East Beltline, Grand Rapids</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>(616) 724-2620 / (616) 364-8214</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Brand store</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>~$7 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Pack size</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Per unit</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="4" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Koeze direct 6-jar case (sale)</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>6 × 17 oz</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>$41.95</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>≈ $6.99/jar</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>CHEAPEST + shipping</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>https://koeze.com/cream-nut-smooth-case-small</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>ShopRite (online listing)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>17 oz</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>$7.39–$7.49</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>$7.39–$7.49/jar</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Out of state; Michigan grocery price likely similar</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>https://www.shoprite.com/sm/pickup/rsid/584/product/creamnut-smooth-natural-peanut-butter-17-oz-id-00071157303412</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>Here Here Market</t>
+          <t>ShopRite (online listing)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4875,47 +4894,79 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>$7.49</t>
+          <t>$7.39–$7.49</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>$7.49/jar</t>
+          <t>$7.39–$7.49/jar</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Out of state; Michigan grocery price likely similar</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://hereheremarket.com/products/cream-nut-natural-peanut-butter-smooth</t>
+          <t>https://www.shoprite.com/sm/pickup/rsid/584/product/creamnut-smooth-natural-peanut-butter-17-oz-id-00071157303412</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
+          <t>Here Here Market</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>17 oz</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>$7.49</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>$7.49/jar</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://hereheremarket.com/products/cream-nut-natural-peanut-butter-smooth</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Harney &amp; Sons</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>17 oz</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>$7.95</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>$7.95/jar</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Free US shipping</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>https://www.harney.com/en-gb/products/koeze-cream-nut-peanut-butter</t>
         </is>
@@ -5614,7 +5665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5689,87 +5740,95 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Meijer – Royal Oak</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>5150 Coolidge Hwy, Royal Oak 48073</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>(248) 280-1800</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Grocery</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Brand on meijer.com</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Meijer lists Pop Daddy (Yellow Mustard, out of stock online). Dill Pickle not seen; check the app.</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>https://www.meijer.com/shopping/product/pop-daddy-yellow-mustard-seasoned-pretzels/85520600528.html</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>~$4–$5 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Pop Daddy direct – 7.5 oz Dill Pickle CASE</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>HQ: 5775 Brighton Pines Ct, Howell</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>(734) 550-9900</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Ship / wholesale</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Case $100; single bags $5.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>https://popdaddysnacks.com/pages/pop-daddy-for-wholesalers</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>$5 single · $100 case</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Market Square (former Papa Joe’s)</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>34244 Woodward Ave, Birmingham, MI 48009</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Pop Daddy locator</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>10 PD items · also Germack</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
@@ -5779,12 +5838,12 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Mkt Square(Birm)Special</t>
+          <t>Market Square (former Papa Joe’s)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>1964 Southfield Rd, Birmingham, MI 48009</t>
+          <t>34244 Woodward Ave, Birmingham, MI 48009</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
@@ -5803,7 +5862,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>6 PD items · also Germack</t>
+          <t>10 PD items · also Germack</t>
         </is>
       </c>
       <c r="I5" s="6" t="n"/>
@@ -5819,12 +5878,12 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>KROGER</t>
+          <t>Mkt Square(Birm)Special</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>685 E Maple Road, Birmingham, MI 48009</t>
+          <t>1964 Southfield Rd, Birmingham, MI 48009</t>
         </is>
       </c>
       <c r="D6" s="6" t="n">
@@ -5843,7 +5902,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>4 PD items</t>
+          <t>6 PD items · also Germack</t>
         </is>
       </c>
       <c r="I6" s="6" t="n"/>
@@ -5864,11 +5923,11 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>1237 Coolidge Highway, Troy, MI 48084</t>
+          <t>685 E Maple Road, Birmingham, MI 48009</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>1.9</v>
+        <v>0.2</v>
       </c>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="inlineStr">
@@ -5894,45 +5953,42 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Walmart</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2001 W Maple Rd, Troy, MI 48084</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>KROGER</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>1237 Coolidge Highway, Troy, MI 48084</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>248-435-4035</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2 PD items</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>~$3–$5 (est.)</t>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>4 PD items</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
@@ -5942,17 +5998,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Naked Fuel</t>
+          <t>Walmart</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2976 W Maple Road, Troy, MI 48084</t>
+          <t>2001 W Maple Rd, Troy, MI 48084</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v>1.9</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>248-435-4035</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>Stockist</t>
@@ -5965,248 +6026,248 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>2 PD items</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>~$3–$5 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Naked Fuel</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2976 W Maple Road, Troy, MI 48084</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Pop Daddy locator</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>1 PD items</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Mkt Fresh</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>31201 Southfield Rd, Beverly hills, MI 48025</t>
         </is>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D11" s="6" t="n">
         <v>2.7</v>
       </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>6 PD items · also Germack</t>
         </is>
       </c>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Michigan Beer Growler Company</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>31221 Southfield Rd, Beverly hills, MI 48025</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>2.7</v>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>1 PD items</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Westborn Market</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>27659 Woodward Avenue, Berkley, MI 48072</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D13" s="6" t="n">
         <v>3.2</v>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>(248) 547-1000</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>13 PD items · also Germack</t>
         </is>
       </c>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>The Neighbor's Shoppe</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>2833 W. 12 Mile Road, Berkley, MI 48072</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D14" t="n">
         <v>3.2</v>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>2 PD items</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Westborn(Berk)Grocery</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>27659 Woodward Ave, Berkley, MI 48072</t>
         </is>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D15" s="6" t="n">
         <v>3.2</v>
       </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>1 PD items · also Germack</t>
         </is>
       </c>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>~$4.50–$6 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Barrel's &amp; Vines Shell</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>31786 Woodward, Royal oak, MI 48073</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Pop Daddy locator</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>7 PD items</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -6218,12 +6279,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KROGER</t>
+          <t>Barrel's &amp; Vines Shell</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>19855 W 12 Mile Road, Southfield, MI 48076</t>
+          <t>31786 Woodward, Royal oak, MI 48073</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -6241,170 +6302,170 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
+          <t>7 PD items</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>~$4.50–$6 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>KROGER</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>19855 W 12 Mile Road, Southfield, MI 48076</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Pop Daddy locator</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>4 PD items</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Plum Market</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>3675 West Maple Road, Bloomfield township, MI 48301</t>
         </is>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D18" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>(248) 594-2555</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>16 PD items · also Germack</t>
         </is>
       </c>
-      <c r="I17" s="6" t="n"/>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>KROGER</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>3600 W Maple Rd, Bloomfield hills, MI 48301</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D19" t="n">
         <v>3.5</v>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>2 PD items</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Nino's (Troy) - Grocery</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>6835 Rochester Rd, Troy, MI 48098</t>
         </is>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D20" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>3 PD items</t>
         </is>
       </c>
-      <c r="I19" s="6" t="n"/>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>~$4.50–$6 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Monarch Market Cafe</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>10099 W Eleven Mile Rd, Huntington woods, MI 48070</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Pop Daddy locator</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>3 PD items</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -6416,77 +6477,71 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>Monarch Market Cafe</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>10099 W Eleven Mile Rd, Huntington woods, MI 48070</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Pop Daddy locator</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>3 PD items</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>~$4.50–$6 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>KROGER</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>3125 John R Road, Troy, MI 48083</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D22" t="n">
         <v>5</v>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>4 PD items</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>~$4.50–$6 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Hollywood Markets</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>714 N Main Street, Royal oak, MI 48067</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>(248) 548-5051</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Pop Daddy locator</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>10 PD items · also Germack</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="n"/>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -6498,18 +6553,22 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Hollywood</t>
+          <t>Hollywood Markets</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>714 N. Main, Royal oak, MI 48067</t>
+          <t>714 N Main Street, Royal oak, MI 48067</t>
         </is>
       </c>
       <c r="D23" s="6" t="n">
         <v>5.4</v>
       </c>
-      <c r="E23" s="6" t="n"/>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>(248) 548-5051</t>
+        </is>
+      </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Stockist</t>
@@ -6522,7 +6581,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>7 PD items · also Germack</t>
+          <t>10 PD items · also Germack</t>
         </is>
       </c>
       <c r="I23" s="6" t="n"/>
@@ -6533,38 +6592,40 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>KROGER</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>2200 E. 12 Mile Road, Royal oak, MI 48067</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Hollywood</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>714 N. Main, Royal oak, MI 48067</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
         <v>5.4</v>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>4 PD items</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>7 PD items · also Germack</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="n"/>
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -6576,12 +6637,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Signature Collective</t>
+          <t>KROGER</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>137 S. Wilson Royal, Oak, MI 48067</t>
+          <t>2200 E. 12 Mile Road, Royal oak, MI 48067</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -6599,7 +6660,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1 PD items</t>
+          <t>4 PD items</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -6614,16 +6675,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>KROGER</t>
+          <t>Signature Collective</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>26200 Greenfield Road, Oak park, MI 48237</t>
+          <t>137 S. Wilson Royal, Oak, MI 48067</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>5.7</v>
+        <v>5.4</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -6637,7 +6698,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>4 PD items</t>
+          <t>1 PD items</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -6657,72 +6718,66 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>26200 Greenfield Road, Oak park, MI 48237</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Pop Daddy locator</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>4 PD items</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>~$4.50–$6 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>KROGER</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>31 E Long Lake Rd, Troy, MI 48085</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D28" t="n">
         <v>6</v>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>3 PD items</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>~$4.50–$6 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Hollywood Markets</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>29200 North Campbell Road, Madison heights, MI 48071</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>(248) 399-0900</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Pop Daddy locator</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>8 PD items · also Germack</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="n"/>
-      <c r="J28" s="6" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
@@ -6734,18 +6789,22 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Hollywood</t>
+          <t>Hollywood Markets</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>29200 Campbell Rd, Madison heights, MI 48071</t>
+          <t>29200 North Campbell Road, Madison heights, MI 48071</t>
         </is>
       </c>
       <c r="D29" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="E29" s="6" t="n"/>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>(248) 399-0900</t>
+        </is>
+      </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Stockist</t>
@@ -6758,7 +6817,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>6 PD items · also Germack</t>
+          <t>8 PD items · also Germack</t>
         </is>
       </c>
       <c r="I29" s="6" t="n"/>
@@ -6769,45 +6828,42 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Costco</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>30550 Stephenson Highway, Madison heights, MI 48071</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Hollywood</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>29200 Campbell Rd, Madison heights, MI 48071</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
         <v>6.3</v>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>(248) 616-0048</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>1 PD items</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>~$3–$5 (est.)</t>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>6 PD items · also Germack</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="n"/>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
@@ -6817,16 +6873,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dd Essentials</t>
+          <t>Costco</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1008 Orchard Ave, Ferndale, MI 48220</t>
+          <t>30550 Stephenson Highway, Madison heights, MI 48071</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>7.2</v>
+        <v>6.3</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>(248) 616-0048</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -6840,12 +6901,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>4 PD items</t>
+          <t>1 PD items</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>~$4.50–$6 (est.)</t>
+          <t>~$3–$5 (est.)</t>
         </is>
       </c>
     </row>
@@ -6855,12 +6916,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>KROGER</t>
+          <t>Dd Essentials</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>8920 W 8 Mile Road, Royal oak twp., MI 48220</t>
+          <t>1008 Orchard Ave, Ferndale, MI 48220</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -6893,22 +6954,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Western Market</t>
+          <t>KROGER</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>447 W Nine Mile Rd, Ferndale, MI 48220</t>
+          <t>8920 W 8 Mile Road, Royal oak twp., MI 48220</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>7.2</v>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>(248) 546-7288</t>
-        </is>
-      </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>Stockist</t>
@@ -6921,7 +6977,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>4 PD items · also Germack</t>
+          <t>4 PD items</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -6936,16 +6992,21 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>KROGER</t>
+          <t>Western Market</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>28250 Dequindre Road, Warren, MI 48092</t>
+          <t>447 W Nine Mile Rd, Ferndale, MI 48220</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>7.8</v>
+        <v>7.2</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>(248) 546-7288</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -6959,7 +7020,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>4 PD items</t>
+          <t>4 PD items · also Germack</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -6979,7 +7040,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>31200 Schoenherr Road, Warren, MI 48092</t>
+          <t>28250 Dequindre Road, Warren, MI 48092</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -7012,22 +7073,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Sheetz</t>
+          <t>KROGER</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>5920 12 Mile Rd, Warren, MI 48092</t>
+          <t>31200 Schoenherr Road, Warren, MI 48092</t>
         </is>
       </c>
       <c r="D36" t="n">
         <v>7.8</v>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>(586) 434-4349</t>
-        </is>
-      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>Stockist</t>
@@ -7040,7 +7096,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2 PD items</t>
+          <t>4 PD items</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -7055,17 +7111,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Simon Express Market&amp;Meal</t>
+          <t>Sheetz</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>31025 Ryan Road, Warren, MI 48092</t>
+          <t>5920 12 Mile Rd, Warren, MI 48092</t>
         </is>
       </c>
       <c r="D37" t="n">
         <v>7.8</v>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>(586) 434-4349</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>Stockist</t>
@@ -7078,7 +7139,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1 PD items</t>
+          <t>2 PD items</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -7093,16 +7154,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KROGER</t>
+          <t>Simon Express Market&amp;Meal</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23101 John R Road, Hazel park, MI 48030</t>
+          <t>31025 Ryan Road, Warren, MI 48092</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>8.300000000000001</v>
+        <v>7.8</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -7116,7 +7177,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>4 PD items</t>
+          <t>1 PD items</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -7136,190 +7197,229 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
+          <t>23101 John R Road, Hazel park, MI 48030</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Pop Daddy locator</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>4 PD items</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>~$4.50–$6 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>KROGER</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
           <t>25780 Middlebelt Road, Farmington hills, MI 48336</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D40" t="n">
         <v>9.6</v>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Stockist</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Stockist</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
         <is>
           <t>Pop Daddy locator</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>4 PD items</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>~$4.50–$6 (est.)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="2" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Pack size</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>Per unit</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="4" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>World Market</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>7.5 oz</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>$4.79</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>$4.79/bag</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>CHEAPEST retail found</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr">
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>https://www.worldmarket.com/p/pop-daddy-dill-pickle-pretzel-sticks-636887.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Pop Daddy direct, single</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>7.5 oz</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>$5.00</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>$5.00/bag</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>https://popdaddysnacks.com/products/pop-daddy-dill-pickle-seasoned-pretzels-7-5oz</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>Provisions co-op wholesale</t>
+          <t>Pop Daddy direct, single</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>case of 12</t>
+          <t>7.5 oz</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>$3.40/bag</t>
+          <t>$5.00</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>$3.40/bag</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Co-op members only; shows what wholesale costs</t>
+          <t>$5.00/bag</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://featherriver.provisions.coop/products/pop-daddy-dill-pickle-4293-9tymax</t>
+          <t>https://popdaddysnacks.com/products/pop-daddy-dill-pickle-seasoned-pretzels-7-5oz</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
+          <t>Provisions co-op wholesale</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>case of 12</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>$3.40/bag</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>$3.40/bag</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Co-op members only; shows what wholesale costs</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://featherriver.provisions.coop/products/pop-daddy-dill-pickle-4293-9tymax</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
           <t>Pop Daddy direct “CASE”</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>≈12 bags (by weight)</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>$100.00</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>≈ $8.33/bag</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>AVOID: costs more per bag than buying singles</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>https://popdaddysnacks.com/pages/pop-daddy-for-wholesalers</t>
         </is>
@@ -8065,7 +8165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8145,76 +8245,81 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
+          <t>Meijer – Royal Oak</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>5150 Coolidge Hwy, Royal Oak 48073</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>(248) 280-1800</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Grocery</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>On meijer.com</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Rock &amp; Rye listed: 2-liter ~$1.69–1.79, Faygo 8-pk 12 oz cans ~$3.99 + deposit.</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>https://www.meijer.com/shopping/product/faygo-rock-rye-67-6-oz-bottle/7380000103.html</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>~$0.50/can in 8-pk (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
           <t>Kroger</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>685 E Maple Rd, Birmingham</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D4" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Grocery</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>~$1–$1.25/can in 12-pk (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>The Detroit Shoppe</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Somerset Collection, 2800 W Big Beaver Rd, Troy</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Gift shop</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Reported</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Carries 7 Faygo flavors.</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>https://www.tripadvisor.com/Attraction_Review-g42763-d2639679-Reviews-The_Detroit_Shoppe-Troy_Michigan.html</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>~$2–$3/can (est.)</t>
         </is>
       </c>
     </row>
@@ -8224,111 +8329,119 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Walmart Troy</t>
+          <t>The Detroit Shoppe</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2001 W Maple Rd, Troy</t>
+          <t>Somerset Collection, 2800 W Big Beaver Rd, Troy</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>1.9</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Gift shop</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Reported</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Carries 7 Faygo flavors.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.tripadvisor.com/Attraction_Review-g42763-d2639679-Reviews-The_Detroit_Shoppe-Troy_Michigan.html</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>~$2–$3/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Walmart Troy</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2001 W Maple Rd, Troy</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>248-435-4035</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Big box</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Listed online</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Rock &amp; Rye 12-pack 12 oz cans.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>~$1/can in store (est.)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Kroger</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>1237 Coolidge Hwy, Troy</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D7" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Grocery</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Likely</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>~$1–$1.25/can in 12-pk (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Faygo store locator</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Locator</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Official</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://www.faygo.com/store-locator</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
@@ -8338,76 +8451,75 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Faygo store locator</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Locator</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.faygo.com/store-locator</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Faygo Beverages HQ &amp; plant</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>3579 Gratiot Ave, Detroit</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>16</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>(313) 925-1600</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Direct (ask)</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>HQ</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Ask about buying cases direct; no public counter confirmed.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Ask</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Beverage Warehouse</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>31111 Greenfield, Beverly Hills MI 48009</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>~$1.50–$2.50/can (est.)</t>
         </is>
       </c>
     </row>
@@ -8417,16 +8529,16 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Troy Cheese &amp; Wine Barn</t>
+          <t>Beverage Warehouse</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>2558 E. Maple, Troy MI 48084</t>
+          <t>31111 Greenfield, Beverly Hills MI 48009</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1.9</v>
+        <v>0.2</v>
       </c>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="inlineStr">
@@ -8453,16 +8565,16 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>BLOOMFIELD MOBIL</t>
+          <t>Troy Cheese &amp; Wine Barn</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
+          <t>2558 E. Maple, Troy MI 48084</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>3.1</v>
+        <v>1.9</v>
       </c>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="inlineStr">
@@ -8489,16 +8601,16 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Campbell Party Store</t>
+          <t>BLOOMFIELD MOBIL</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>3321 Campbell, Royal Oak MI 48073</t>
+          <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="inlineStr">
@@ -8525,16 +8637,16 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>MOBIL - TELEGRAPH</t>
+          <t>Campbell Party Store</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>6490 TELEGRAPH RD, BLOOMFIELD HILLS MI 48301</t>
+          <t>3321 Campbell, Royal Oak MI 48073</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="inlineStr">
@@ -8561,12 +8673,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Shell _Bloomfield - Barbat</t>
+          <t>MOBIL - TELEGRAPH</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>3690 W Maple, West Bloomfiled MI 48301</t>
+          <t>6490 TELEGRAPH RD, BLOOMFIELD HILLS MI 48301</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
@@ -8597,16 +8709,16 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Manny's Liquor</t>
+          <t>Shell _Bloomfield - Barbat</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>42951 Dequindre, Troy MI 48098</t>
+          <t>3690 W Maple, West Bloomfiled MI 48301</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="inlineStr">
@@ -8633,16 +8745,16 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Bloomfield Wine &amp; Spirits</t>
+          <t>Manny's Liquor</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>1081 W. Long Lake Road, Bloomfield Hills MI 48302</t>
+          <t>42951 Dequindre, Troy MI 48098</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="inlineStr">
@@ -8663,99 +8775,136 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Bloomfield Wine &amp; Spirits</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>1081 W. Long Lake Road, Bloomfield Hills MI 48302</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>~$1.50–$2.50/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Pack size</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Per unit</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Kroger / Meijer in-store 12-pack</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>12 × 12 oz</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>check app</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Likely cheapest; no posted price found. Check the Kroger app for 685 E Maple.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
+          <t>Kroger / Meijer in-store 12-pack</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>12 × 12 oz</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>check app</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Likely cheapest; no posted price found. Check the Kroger app for 685 E Maple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
           <t>Walmart marketplace 12-pack</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>12 × 12 oz</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>≈ $24.47</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>≈ $2.04/can</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Marked-up third-party seller; avoid</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>https://www.walmart.com/ip/seort/631284437</t>
         </is>

</xml_diff>

<commit_message>
Add shopping plan tab and correct box size to 16x12x8
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SS8EsZNZJgzhYPJLGv3Rn9
</commit_message>
<xml_diff>
--- a/Michigan_Box_By_Item.xlsx
+++ b/Michigan_Box_By_Item.xlsx
@@ -7,16 +7,17 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shipping" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Cherries" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Fudge" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Cream-Nut" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Peanuts" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Pretzels" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Kars" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Faygo" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Card" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shopping Plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shipping" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Cherries" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Fudge" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Cream-Nut" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Peanuts" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Pretzels" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Kars" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Faygo" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Card" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -77,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -89,6 +90,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -454,7 +458,659 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:G34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>SHOPPING PLAN – 1 Michigan Box, from Birmingham MI. Call Market Square and Germack first. If Germack isn’t nearby, the Eastern Market shop (2509 Russell St) closes at 3 PM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Buy at</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Backup</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Est. price</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Est. weight (oz)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Got it?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Germack Dried Michigan Cherries, 8 oz</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Market Square, 34244 Woodward, Birmingham</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Germack store, 2509 Russell St, Detroit (closes 3 PM)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>~$14</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mackinac Island Fudge (Devon’s 7 oz tub)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ace Hardware, 17670 13 Mile, Beverly Hills</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ace Clawson 149 E 14 Mile · Ace Royal Oak 515 E 4th</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>~$5</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Koeze Cream-Nut Peanut Butter, 17 oz</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Meijer, 5150 Coolidge Hwy, Royal Oak</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Kroger, 685 E Maple, Birmingham</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>~$6–7.50</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Germack In-Shell Peanuts (7 oz online; 9 oz not found)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Market Square, 34244 Woodward</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Germack store, Eastern Market</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>~$4–5</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pop Daddy Dill Pickle Pretzels, 7.5 oz</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Market Square, 34244 Woodward</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Plum Market, 3675 W Maple, Bloomfield</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>~$5</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Kar’s Sweet ’N Salty, 2 oz</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Market Square or Meijer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Kroger, 685 E Maple</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>~$1–1.50</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Faygo Rock &amp; Rye, 12 oz can</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Meijer, 5150 Coolidge Hwy, Royal Oak</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Kroger, 685 E Maple</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>~$1–2</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>13</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Greetings from Detroit Card, 5×7</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FedEx Office, 33100 Woodward (print) + envelope at Paper Source, 115 W Maple</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>The UPS Store, 33717 Woodward</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>~$5–10</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>ITEMS TOTAL</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>≈ $42–50</t>
+        </is>
+      </c>
+      <c r="F12">
+        <f>SUM(F4:F11)</f>
+        <v/>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>≈ 4.8 lb</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>PACKAGING</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Magnetic gift box, about 13.5 × 10 × 5 in inside</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>The Container Store, 2805 E Big Beaver, Troy, (248) 859-7320</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Michaels, 1205 Coolidge Hwy, Troy</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>~$25–30</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>~1.2 lb</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Shipping box 16 × 12 × 8 in</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FedEx Office, 33100 Woodward</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>The UPS Store, 33717 Woodward</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>~$5</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>~0.9 lb</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Crinkle filler, tissue, tape, zip bag (for can)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Dollar Tree, 33877 Woodward (if open)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Paper Source, 115 W Maple</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>~$5</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>~0.4 lb</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FedEx Office, 33100 Woodward: order the card print</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Dollar Tree, 33877 Woodward: filler, tape, zip bag</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Market Square, 34244 Woodward: items 1, 4, 5, 6</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Paper Source, 115 W Maple: envelope, tissue</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>The Container Store, Troy (or Michaels): gift box. Test-fit the items.</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Meijer, Royal Oak: items 3, 7</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ace Hardware, Beverly Hills: item 2</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>FedEx Office: pick up the card, buy the 16×12×8 box, pack, weigh, ship</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>SHIPPING SCREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Length × Width × Height</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16 × 12 × 8 in</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Weight (empty)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2.5 lb</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Total weight</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8 lb (or the real weight from the FedEx scale)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>USPS Ground Advantage</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Shopify product weight</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>4.8 lb</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -466,14 +1122,13 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="52" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="60" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Michigan Box: one tab per item, sorted nearest to Birmingham, MI (48009) first. Stockist rows come from the brands’ official store locators (pulled 10/26/2026). Those list stores carrying the brand, not the exact bag, so call ahead. Prices come from public listings and may change. Each item tab ends with a PRICE COMPARISON table (cheapest first, highlighted green). "Est. price" = a price found in a listing, or "(est.)" where it is an estimate. Confirm in store. PURPLE rows = the same place appears in 2+ other item tabs (one stop for several items). Meijer Royal Oak (5150 Coolidge Hwy) added: confirmed online for Cream-Nut and Faygo Rock &amp; Rye.</t>
+          <t>Faygo Rock &amp; Rye, 12 oz can. Widely stocked. Use the Faygo store locator (choose Rock &amp; Rye, enter 48009) to confirm a store.</t>
         </is>
       </c>
     </row>
@@ -525,103 +1180,91 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Est. price (cheapest option)</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Est. item weight (with its own packaging)</t>
+          <t>Est. price</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Germack Dried Cherries 8 oz → tab "1 Cherries"</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Market Square, 34244 Woodward (former Papa Joe’s) or 1964 Southfield Rd</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Meijer – Royal Oak</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>5150 Coolidge Hwy, Royal Oak 48073</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>(248) 280-1800</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Grocery</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>On meijer.com</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Rock &amp; Rye listed: 2-liter ~$1.69–1.79, Faygo 8-pk 12 oz cans ~$3.99 + deposit.</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>https://www.meijer.com/shopping/product/faygo-rock-rye-67-6-oz-bottle/7380000103.html</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>~$0.50/can in 8-pk (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Kroger</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>685 E Maple Rd, Birmingham</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Best Birmingham stop</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Germack stockist</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Surest source: Germack’s Eastern Market shop (16.6 mi)</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Germack 8 oz $14.24 (online/store)</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>8.4 oz (8 oz net)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Mackinac Island Fudge 8 oz → tab "2 Fudge"</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Ace Hardware, 17670 13 Mile Rd, Beverly Hills (Devon’s Mackinac Island Fudge)</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>(906) 643-9616 Murdick’s business</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Best nearby stop</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Ace sells Devon’s; call to confirm</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>7 oz tub. Clawson, Southfield and Royal Oak Aces too. Ship from Joann’s if none in stock.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>$4.99 (7 oz tub)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>9.0 oz (8 oz net)</t>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Grocery</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>~$1–$1.25/can in 12-pk (est.)</t>
         </is>
       </c>
     </row>
@@ -631,50 +1274,40 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Koeze Cream-Nut 17 oz → tab "3 Cream-Nut"</t>
+          <t>The Detroit Shoppe</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Meijer, 5150 Coolidge Hwy, Royal Oak (listed on meijer.com)</t>
+          <t>Somerset Collection, 2800 W Big Beaver Rd, Troy</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>(616) 724-2620</t>
-        </is>
+        <v>1.9</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Best nearby stop</t>
+          <t>Gift shop</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>On meijer.com</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Check Kroger, 685 E Maple on kroger.com</t>
+          <t>Carries 7 Faygo flavors.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://koeze.com/cream-nut-smooth-case-small</t>
+          <t>https://www.tripadvisor.com/Attraction_Review-g42763-d2639679-Reviews-The_Detroit_Shoppe-Troy_Michigan.html</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>$7.49 ($5.99 sale)</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>26.5 oz (17 oz net)</t>
+          <t>~$2–$3/can (est.)</t>
         </is>
       </c>
     </row>
@@ -684,88 +1317,76 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Germack In-Shell Peanuts 9 oz → tab "4 Peanuts"</t>
+          <t>Walmart Troy</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Market Square (either Birmingham store)</t>
+          <t>2001 W Maple Rd, Troy</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.2</v>
+        <v>1.9</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>248-435-4035</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Best Birmingham stop</t>
+          <t>Big box</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Germack stockist</t>
+          <t>Listed online</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Same stores as the cherries</t>
+          <t>Rock &amp; Rye 12-pack 12 oz cans.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Germack 10 lb bulk $24.99 ≈ $1.40 per 9 oz (7 oz bag $4.25)</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>9.4 oz (9 oz net)</t>
+          <t>~$1/can in store (est.)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Pop Daddy Dill Pickle 7.5 oz → tab "5 Pretzels"</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Market Square, 34244 Woodward (10 Pop Daddy items listed)</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Best Birmingham stop</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Pop Daddy stockist</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Case of 7.5 oz Dill Pickle direct: $100</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://popdaddysnacks.com/pages/pop-daddy-for-wholesalers</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Single bags ~$4.79–$5 (skip the $100 case)</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>8.0 oz (7.5 oz net)</t>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Kroger</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>1237 Coolidge Hwy, Troy</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Grocery</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>~$1–$1.25/can in 12-pk (est.)</t>
         </is>
       </c>
     </row>
@@ -775,50 +1396,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kar’s Sweet ’N Salty 2 oz → tab "6 Kars"</t>
+          <t>Faygo store locator</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Costco, 30550 Stephenson Hwy, Madison Hts</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>(248) 616-0048</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Bulk</t>
+          <t>Locator</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Online listing</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>24 ct × 2 oz ≈ $11; singles at Kroger 685 E Maple</t>
+          <t>Official</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://www.costco.com/.product.411389.html</t>
+          <t>https://www.faygo.com/store-locator</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Sam’s Club 40-pk $17.48 ≈ $0.44/bag</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>2.2 oz (2 oz net)</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -828,92 +1431,429 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Faygo Rock &amp; Rye 12 oz → tab "7 Faygo"</t>
+          <t>Faygo Beverages HQ &amp; plant</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kroger, 685 E Maple, Birmingham</t>
+          <t>3579 Gratiot Ave, Detroit</t>
         </is>
       </c>
       <c r="D9" t="n">
+        <v>16</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>(313) 925-1600</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Direct (ask)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Ask about buying cases direct; no public counter confirmed.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Beverage Warehouse</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>31111 Greenfield, Beverly Hills MI 48009</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Grocery</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Widely stocked</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Use the Faygo locator to confirm the flavor</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>https://www.faygo.com/store-locator</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>In-store Kroger/Meijer 12-pack (skip online ~$24)</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>13.0 oz (12 fl oz net)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Greetings from Detroit Card → tab "8 Card"</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Paper Source, 115 W Maple, Birmingham</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Stationery</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Listed</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>For Detroit-artist cards: City Bird, Midtown Detroit</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Custom print run (get quotes)</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>1.0 oz (5×7 in net)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>~$1.50–$2.50/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Troy Cheese &amp; Wine Barn</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>2558 E. Maple, Troy MI 48084</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>~$1.50–$2.50/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>BLOOMFIELD MOBIL</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>~$1.50–$2.50/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Campbell Party Store</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>3321 Campbell, Royal Oak MI 48073</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>~$1.50–$2.50/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>MOBIL - TELEGRAPH</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>6490 TELEGRAPH RD, BLOOMFIELD HILLS MI 48301</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>~$1.50–$2.50/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Shell _Bloomfield - Barbat</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>3690 W Maple, West Bloomfiled MI 48301</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>~$1.50–$2.50/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Manny's Liquor</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>42951 Dequindre, Troy MI 48098</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>~$1.50–$2.50/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Bloomfield Wine &amp; Spirits</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>1081 W. Long Lake Road, Bloomfield Hills MI 48302</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>~$1.50–$2.50/can (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Pack size</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Per unit</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Kroger / Meijer in-store 12-pack</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>12 × 12 oz</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>check app</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Likely cheapest; no posted price found. Check the Kroger app for 685 E Maple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Walmart marketplace 12-pack</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>12 × 12 oz</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>≈ $24.47</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>≈ $2.04/can</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Marked-up third-party seller; avoid</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.walmart.com/ip/seort/631284437</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
@@ -922,7 +1862,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1333,6 +2273,479 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="60" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The Michigan Box: one tab per item, sorted nearest to Birmingham, MI (48009) first. Stockist rows come from the brands’ official store locators (pulled 10/26/2026). Those list stores carrying the brand, not the exact bag, so call ahead. Prices come from public listings and may change. Each item tab ends with a PRICE COMPARISON table (cheapest first, highlighted green). "Est. price" = a price found in a listing, or "(est.)" where it is an estimate. Confirm in store. PURPLE rows = the same place appears in 2+ other item tabs (one stop for several items). Meijer Royal Oak (5150 Coolidge Hwy) added: confirmed online for Cream-Nut and Faygo Rock &amp; Rye.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Place</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Miles from Birmingham</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Est. price (cheapest option)</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Est. item weight (with its own packaging)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Germack Dried Cherries 8 oz → tab "1 Cherries"</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Market Square, 34244 Woodward (former Papa Joe’s) or 1964 Southfield Rd</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Best Birmingham stop</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Germack stockist</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Surest source: Germack’s Eastern Market shop (16.6 mi)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Germack 8 oz $14.24 (online/store)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>8.4 oz (8 oz net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mackinac Island Fudge 8 oz → tab "2 Fudge"</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ace Hardware, 17670 13 Mile Rd, Beverly Hills (Devon’s Mackinac Island Fudge)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>(906) 643-9616 Murdick’s business</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Best nearby stop</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Ace sells Devon’s; call to confirm</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>7 oz tub. Clawson, Southfield and Royal Oak Aces too. Ship from Joann’s if none in stock.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>$4.99 (7 oz tub)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>9.0 oz (8 oz net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Koeze Cream-Nut 17 oz → tab "3 Cream-Nut"</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Meijer, 5150 Coolidge Hwy, Royal Oak (listed on meijer.com)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>(616) 724-2620</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Best nearby stop</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>On meijer.com</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Check Kroger, 685 E Maple on kroger.com</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://koeze.com/cream-nut-smooth-case-small</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>$7.49 ($5.99 sale)</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>26.5 oz (17 oz net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Germack In-Shell Peanuts 9 oz → tab "4 Peanuts"</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Market Square (either Birmingham store)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Best Birmingham stop</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Germack stockist</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Same stores as the cherries</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Germack 10 lb bulk $24.99 ≈ $1.40 per 9 oz (7 oz bag $4.25)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>9.4 oz (9 oz net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pop Daddy Dill Pickle 7.5 oz → tab "5 Pretzels"</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Market Square, 34244 Woodward (10 Pop Daddy items listed)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Best Birmingham stop</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pop Daddy stockist</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Case of 7.5 oz Dill Pickle direct: $100</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://popdaddysnacks.com/pages/pop-daddy-for-wholesalers</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Single bags ~$4.79–$5 (skip the $100 case)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>8.0 oz (7.5 oz net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kar’s Sweet ’N Salty 2 oz → tab "6 Kars"</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Costco, 30550 Stephenson Hwy, Madison Hts</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>(248) 616-0048</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Bulk</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Online listing</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>24 ct × 2 oz ≈ $11; singles at Kroger 685 E Maple</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.costco.com/.product.411389.html</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Sam’s Club 40-pk $17.48 ≈ $0.44/bag</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2.2 oz (2 oz net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Faygo Rock &amp; Rye 12 oz → tab "7 Faygo"</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Kroger, 685 E Maple, Birmingham</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Grocery</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Widely stocked</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Use the Faygo locator to confirm the flavor</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.faygo.com/store-locator</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>In-store Kroger/Meijer 12-pack (skip online ~$24)</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>13.0 oz (12 fl oz net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Greetings from Detroit Card → tab "8 Card"</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Paper Source, 115 W Maple, Birmingham</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Stationery</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Listed</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>For Detroit-artist cards: City Bird, Midtown Detroit</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Custom print run (get quotes)</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1.0 oz (5×7 in net)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1350,6 +2763,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1571,11 +2985,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Gift box + shipping box + filler (est.)</t>
+          <t>Magnetic gift box + shipping box + filler (est.)</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1598,6 +3012,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -1630,7 +3045,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>12 × 10 × 6 in (or 12 × 9 × 6)</t>
+          <t>16 × 12 × 8 in (gift box ~13.5 × 10 × 5 inside)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1647,12 +3062,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>12×10×6 = 720 in³ ÷ 139 ≈ 5.2 lb</t>
+          <t>16×12×8 = 1,536 in³ ÷ 139 ≈ 11 lb</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Lower than the actual ~6.1 lb, so you are billed on actual weight</t>
+          <t>Higher than the actual ~7.3 lb, so UPS/FedEx bill ~11 lb. Use USPS.</t>
         </is>
       </c>
     </row>
@@ -1669,7 +3084,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Billed on actual weight, rounded up to the next lb (≈ 7 lb)</t>
+          <t>Under 1,728 in³, so billed on actual weight, rounded up (≈ 8 lb)</t>
         </is>
       </c>
     </row>
@@ -1681,7 +3096,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Box, 12 × 10 × 6 in, total ≈ 6.1 lb (confirm on a scale)</t>
+          <t>Box, 16 × 12 × 8 in, empty 2.5 lb, total ≈ 8 lb (confirm on a scale)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1698,7 +3113,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3642,7 +5057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4398,7 +5813,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4809,7 +6224,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -4980,7 +6394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5659,7 +7073,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7262,7 +8676,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
@@ -7422,732 +8835,6 @@
       <c r="G47" t="inlineStr">
         <is>
           <t>https://popdaddysnacks.com/pages/pop-daddy-for-wholesalers</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="60" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Kar’s Sweet ’N Salty, 2 oz. Costco sells the 24-count box. Single bags are at most groceries and party stores; the party stores below are likely, not verified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Place</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Address</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Miles from Birmingham</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Confidence</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Est. price</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Costco Madison Heights</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>30550 Stephenson Hwy, Madison Heights</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>(248) 616-0048</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Club / bulk</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Online listing</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>24 ct × 2 oz (item 411389) ≈ $11; check warehouse stock.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://www.costco.com/.product.411389.html</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>≈ $0.46/bag (24-pk ~$11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Kroger</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>685 E Maple Rd, Birmingham</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Grocery</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Single bags.</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>~$1–$1.50 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Kar’s Nuts HQ</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1200 E 14 Mile Rd, Madison Heights</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Wholesale (ask)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>HQ</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>No outlet store confirmed.</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://karsnuts.com</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Wholesale (ask)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Home Depot (online)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Ship to store</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Online bulk</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Listed</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>24-ct caddy ≈ $21.98.</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>https://www.homedepot.com/p/Kar-s-2-oz-Packets-Sweet-N-Salty-Mix-Nuts-Caddy-24-Box-AVTSN08387/320270957</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>≈ $0.92/bag</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Beverage Warehouse</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>31111 Greenfield, Beverly Hills MI 48009</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>~$1–$2 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Troy Cheese &amp; Wine Barn</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>2558 E. Maple, Troy MI 48084</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>~$1–$2 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>BLOOMFIELD MOBIL</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>~$1–$2 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Campbell Party Store</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>3321 Campbell, Royal Oak MI 48073</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>~$1–$2 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>MOBIL - TELEGRAPH</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>6490 TELEGRAPH RD, BLOOMFIELD HILLS MI 48301</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="6" t="n"/>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>~$1–$2 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Shell _Bloomfield - Barbat</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>3690 W Maple, West Bloomfiled MI 48301</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>~$1–$2 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Manny's Liquor</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>42951 Dequindre, Troy MI 48098</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>~$1–$2 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Bloomfield Wine &amp; Spirits</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>1081 W. Long Lake Road, Bloomfield Hills MI 48302</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>~$1–$2 (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Option</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Pack size</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Per unit</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Sam’s Club 40-pack</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>40 × 2 oz</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>$17.48</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>≈ $0.44/bag</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>CHEAPEST</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>https://www.samsclub.com/ip/Kar-s-Sweet-n-Salty-Trail-Mix-2-oz-40-pk/7703408821</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Costco 24-pack (item 411389)</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>24 × 2 oz</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>≈ $10.99–$11.49</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>≈ $0.46/bag</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Third-party price tracker</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://app.warehouserunner.com/costco/411389</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Walmart 24-pack</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>24 × 2 oz</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>$19.99</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>≈ $0.83/bag</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.walmart.com/ip/Kar-s-Nuts-Caddy-Sweet-N-Salty-Mix-2-oz-Packets-24-Box-Each/1857595784</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Home Depot 24-pack</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>24 × 2 oz</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>$21.98</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>≈ $0.92/bag</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Staples 24-pack</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>24 × 2 oz</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>$27.99</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>≈ $1.17/bag</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://www.staples.com/kar-s-gluten-free-sweet-n-salty-snack-mix-2-oz-24-bags-pack-kar08387/product_495720</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8870,7 @@
     <row r="1" ht="60" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Faygo Rock &amp; Rye, 12 oz can. Widely stocked. Use the Faygo store locator (choose Rock &amp; Rye, enter 48009) to confirm a store.</t>
+          <t>Kar’s Sweet ’N Salty, 2 oz. Costco sells the 24-count box. Single bags are at most groceries and party stores; the party stores below are likely, not verified.</t>
         </is>
       </c>
     </row>
@@ -8240,50 +8927,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Meijer – Royal Oak</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>5150 Coolidge Hwy, Royal Oak 48073</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>(248) 280-1800</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Grocery</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>On meijer.com</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>Rock &amp; Rye listed: 2-liter ~$1.69–1.79, Faygo 8-pk 12 oz cans ~$3.99 + deposit.</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>https://www.meijer.com/shopping/product/faygo-rock-rye-67-6-oz-bottle/7380000103.html</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>~$0.50/can in 8-pk (est.)</t>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Costco Madison Heights</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>30550 Stephenson Hwy, Madison Heights</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>(248) 616-0048</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Club / bulk</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Online listing</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>24 ct × 2 oz (item 411389) ≈ $11; check warehouse stock.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.costco.com/.product.411389.html</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>≈ $0.46/bag (24-pk ~$11)</t>
         </is>
       </c>
     </row>
@@ -8315,11 +9002,15 @@
           <t>Likely</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Single bags.</t>
+        </is>
+      </c>
       <c r="I4" s="6" t="n"/>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>~$1–$1.25/can in 12-pk (est.)</t>
+          <t>~$1–$1.50 (est.)</t>
         </is>
       </c>
     </row>
@@ -8329,40 +9020,40 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The Detroit Shoppe</t>
+          <t>Kar’s Nuts HQ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Somerset Collection, 2800 W Big Beaver Rd, Troy</t>
+          <t>1200 E 14 Mile Rd, Madison Heights</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.9</v>
+        <v>6.3</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Gift shop</t>
+          <t>Wholesale (ask)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>HQ</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Carries 7 Faygo flavors.</t>
+          <t>No outlet store confirmed.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.tripadvisor.com/Attraction_Review-g42763-d2639679-Reviews-The_Detroit_Shoppe-Troy_Michigan.html</t>
+          <t>https://karsnuts.com</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>~$2–$3/can (est.)</t>
+          <t>Wholesale (ask)</t>
         </is>
       </c>
     </row>
@@ -8372,40 +9063,37 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Walmart Troy</t>
+          <t>Home Depot (online)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2001 W Maple Rd, Troy</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>248-435-4035</t>
+          <t>Ship to store</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Big box</t>
+          <t>Online bulk</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Listed online</t>
+          <t>Listed</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Rock &amp; Rye 12-pack 12 oz cans.</t>
+          <t>24-ct caddy ≈ $21.98.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.homedepot.com/p/Kar-s-2-oz-Packets-Sweet-N-Salty-Mix-Nuts-Caddy-24-Box-AVTSN08387/320270957</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>~$1/can in store (est.)</t>
+          <t>≈ $0.92/bag</t>
         </is>
       </c>
     </row>
@@ -8415,21 +9103,21 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Kroger</t>
+          <t>Beverage Warehouse</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>1237 Coolidge Hwy, Troy</t>
+          <t>31111 Greenfield, Beverly Hills MI 48009</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>1.9</v>
+        <v>0.2</v>
       </c>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Grocery</t>
+          <t>Party store</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -8441,85 +9129,79 @@
       <c r="I7" s="6" t="n"/>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>~$1–$1.25/can in 12-pk (est.)</t>
+          <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Faygo store locator</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Locator</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Official</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>https://www.faygo.com/store-locator</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Troy Cheese &amp; Wine Barn</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>2558 E. Maple, Troy MI 48084</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Faygo Beverages HQ &amp; plant</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>3579 Gratiot Ave, Detroit</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>16</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>(313) 925-1600</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Direct (ask)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>HQ</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Ask about buying cases direct; no public counter confirmed.</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Ask</t>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>BLOOMFIELD MOBIL</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Party store</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
@@ -8529,16 +9211,16 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Beverage Warehouse</t>
+          <t>Campbell Party Store</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>31111 Greenfield, Beverly Hills MI 48009</t>
+          <t>3321 Campbell, Royal Oak MI 48073</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.2</v>
+        <v>3.4</v>
       </c>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="inlineStr">
@@ -8555,7 +9237,7 @@
       <c r="I10" s="6" t="n"/>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>~$1.50–$2.50/can (est.)</t>
+          <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
@@ -8565,16 +9247,16 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Troy Cheese &amp; Wine Barn</t>
+          <t>MOBIL - TELEGRAPH</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>2558 E. Maple, Troy MI 48084</t>
+          <t>6490 TELEGRAPH RD, BLOOMFIELD HILLS MI 48301</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>1.9</v>
+        <v>3.5</v>
       </c>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="inlineStr">
@@ -8591,7 +9273,7 @@
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>~$1.50–$2.50/can (est.)</t>
+          <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
@@ -8601,16 +9283,16 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>BLOOMFIELD MOBIL</t>
+          <t>Shell _Bloomfield - Barbat</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>1501 SOUTH OPDYKE RD, BLOOMFIELD TWP MI 48304</t>
+          <t>3690 W Maple, West Bloomfiled MI 48301</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="inlineStr">
@@ -8627,7 +9309,7 @@
       <c r="I12" s="6" t="n"/>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>~$1.50–$2.50/can (est.)</t>
+          <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
@@ -8637,16 +9319,16 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Campbell Party Store</t>
+          <t>Manny's Liquor</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>3321 Campbell, Royal Oak MI 48073</t>
+          <t>42951 Dequindre, Troy MI 48098</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="inlineStr">
@@ -8663,7 +9345,7 @@
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>~$1.50–$2.50/can (est.)</t>
+          <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
@@ -8673,16 +9355,16 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>MOBIL - TELEGRAPH</t>
+          <t>Bloomfield Wine &amp; Spirits</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>6490 TELEGRAPH RD, BLOOMFIELD HILLS MI 48301</t>
+          <t>1081 W. Long Lake Road, Bloomfield Hills MI 48302</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="inlineStr">
@@ -8699,214 +9381,186 @@
       <c r="I14" s="6" t="n"/>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>~$1.50–$2.50/can (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Shell _Bloomfield - Barbat</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>3690 W Maple, West Bloomfiled MI 48301</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>~$1.50–$2.50/can (est.)</t>
+          <t>~$1–$2 (est.)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Manny's Liquor</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>42951 Dequindre, Troy MI 48098</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>~$1.50–$2.50/can (est.)</t>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Bloomfield Wine &amp; Spirits</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>1081 W. Long Lake Road, Bloomfield Hills MI 48302</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Party store</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Likely</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>~$1.50–$2.50/can (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pack size</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Per unit</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Sam’s Club 40-pack</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>40 × 2 oz</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>$17.48</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>≈ $0.44/bag</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>CHEAPEST</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.samsclub.com/ip/Kar-s-Sweet-n-Salty-Trail-Mix-2-oz-40-pk/7703408821</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>PRICE COMPARISON (cheapest first, from public listings 10/26/2026; shipping and tax not included)</t>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Costco 24-pack (item 411389)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>24 × 2 oz</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>≈ $10.99–$11.49</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>≈ $0.46/bag</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Third-party price tracker</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://app.warehouserunner.com/costco/411389</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Option</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Pack size</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Per unit</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Link</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Walmart 24-pack</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>24 × 2 oz</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>$19.99</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>≈ $0.83/bag</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.walmart.com/ip/Kar-s-Nuts-Caddy-Sweet-N-Salty-Mix-2-oz-Packets-24-Box-Each/1857595784</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kroger / Meijer in-store 12-pack</t>
+          <t>Home Depot 24-pack</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>12 × 12 oz</t>
+          <t>24 × 2 oz</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>check app</t>
+          <t>$21.98</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Likely cheapest; no posted price found. Check the Kroger app for 685 E Maple.</t>
+          <t>≈ $0.92/bag</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>Walmart marketplace 12-pack</t>
+          <t>Staples 24-pack</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>12 × 12 oz</t>
+          <t>24 × 2 oz</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>≈ $24.47</t>
+          <t>$27.99</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>≈ $2.04/can</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Marked-up third-party seller; avoid</t>
+          <t>≈ $1.17/bag</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/ip/seort/631284437</t>
+          <t>https://www.staples.com/kar-s-gluten-free-sweet-n-salty-snack-mix-2-oz-24-bags-pack-kar08387/product_495720</t>
         </is>
       </c>
     </row>

</xml_diff>